<commit_message>
docs(inventory): record Li-S BMS fastener source conflict
Document the adapted Wickerts Table S26 value (2.8e-3 kg) versus the cited original Ellingsen (2014) detailed BMS value (2.8e-2 kg). Retain the existing 0.028 kg supported by the original inventory. No recipe changes or claim of resolved BMS sizing/coverage.

Scope: existing supplemental workbook inventories only. Approved as item 7 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-batteries-LiS.xlsx
+++ b/premise/data/additional_inventories/lci-batteries-LiS.xlsx
@@ -9993,8 +9993,12 @@
       <c r="A587" t="s">
         <v>1</v>
       </c>
-      <c r="B587" t="s">
-        <v>410</v>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>APPROVED Li-S BMS FASTENER SOURCE-CONFLICT NOTE, 2026-10-18. The adapted Wickerts supporting information Table S26 lists IBIS fasteners at 2.8E-3 kg per BMS inventory, while its cited original Ellingsen et al. (2014) supporting-information detailed BMS component inventory lists IBIS fasteners at 2.8E-2 kg. The original source therefore supports retaining the existing 0.028 kg fastener input (B602). Do not silently reduce it tenfold to match the adapted table. This records an unresolved source conflict; it does not validate complete BMS sizing, module/rack allocation, cooling coverage or metal composition. All BMS quantities and suppliers remain unchanged.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+This activity is aggregated to match the requirements of one battery rack, as it is modelled in the lithium-sulfur study. This includes both the BMS on a module level as well as on the rack level. BMS=battery management system. PCB=printed circut board. Source: Wickerts et al. (2023). Prospective Life Cycle Assessment of Lithium-Sulfur Batteries for Stationary Energy Storage. ACS Sustainable Chemistry &amp; Engineering. https://doi.org/10.1021/acssuschemeng.3c00141</t>
+        </is>
       </c>
     </row>
     <row r="588" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
docs(inventory): distinguish Li-S cell and module reference values
Clarify that the implemented 150 Wh/kg and 225 lifetime kWh/kg refer to cells. Use the unchanged 0.7515918465419887 cell share to document 112.7388 Wh/kg module and 169.1082 lifetime kWh/kg module. Replace the copied 321 kg market-output claim with the existing 1 kg module reference. No quantity or energy-density change; explicitly retain the unresolved mismatch with the 500 Wh/kg source composition.

Scope: existing supplemental workbook inventories only. Approved as item 6 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-batteries-LiS.xlsx
+++ b/premise/data/additional_inventories/lci-batteries-LiS.xlsx
@@ -8700,8 +8700,12 @@
       <c r="A491" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B491" s="16" t="s">
-        <v>413</v>
+      <c r="B491" s="16" t="inlineStr">
+        <is>
+          <t>APPROVED Li-S CELL/MODULE METADATA CLARIFICATION, 2026-10-18. The implemented 150 Wh/kg (0.150 kWh/kg) is a CELL-specific reference, not energy per kg module. The existing module recipe contains 408*0.046/24.971 = 0.7515918465419887 kg cell/kg module, giving 0.1127387769812983 kWh/kg module at that cell reference. At the inherited 1500 cycles, 225 kWh/kg applies to CELL mass; the corresponding reference is 169.10816547194747 kWh/kg MODULE. Market output is 1 kg battery module, not a 321 kg system (that was a copied Li-O2 label). These are explanatory conversions under existing assumptions; no recipe, density trajectory, cycle life, replacement or per-MJ allocation is changed. IMPORTANT UNRESOLVED DESIGN GAP: the Wickerts composition reference uses a 500 Wh/kg cell design, whereas the implemented baseline is 150 Wh/kg; this documentation does not reconcile their physical designs or validate complete BMS/cooling coverage. Historical statements below are retained only as history and the cell/module clarification above takes precedence.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Specific energy density: 150 Wh/kg. Projected up to 500 Wh/kg in an optimistic future || Cycle life: 1500 || Lifetime: 225 kWh/kg.Source: Wickerts et al. (2023). Prospective Life Cycle Assessment of Lithium-Sulfur Batteries for Stationary Energy Storage. ACS Sustainable Chemistry &amp; Engineering. https://doi.org/10.1021/acssuschemeng.3c00141</t>
+        </is>
       </c>
     </row>
     <row r="492" spans="1:7" x14ac:dyDescent="0.2">
@@ -8984,8 +8988,12 @@
       <c r="A510" t="s">
         <v>1</v>
       </c>
-      <c r="B510" s="28" t="s">
-        <v>413</v>
+      <c r="B510" s="28" t="inlineStr">
+        <is>
+          <t>APPROVED Li-S CELL/MODULE METADATA CLARIFICATION, 2026-10-18. The implemented 150 Wh/kg (0.150 kWh/kg) is a CELL-specific reference, not energy per kg module. The existing module recipe contains 408*0.046/24.971 = 0.7515918465419887 kg cell/kg module, giving 0.1127387769812983 kWh/kg module at that cell reference. At the inherited 1500 cycles, 225 kWh/kg applies to CELL mass; the corresponding reference is 169.10816547194747 kWh/kg MODULE. Market output is 1 kg battery module, not a 321 kg system (that was a copied Li-O2 label). These are explanatory conversions under existing assumptions; no recipe, density trajectory, cycle life, replacement or per-MJ allocation is changed. IMPORTANT UNRESOLVED DESIGN GAP: the Wickerts composition reference uses a 500 Wh/kg cell design, whereas the implemented baseline is 150 Wh/kg; this documentation does not reconcile their physical designs or validate complete BMS/cooling coverage. Historical statements below are retained only as history and the cell/module clarification above takes precedence.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Specific energy density: 150 Wh/kg. Projected up to 500 Wh/kg in an optimistic future || Cycle life: 1500 || Lifetime: 225 kWh/kg.Source: Wickerts et al. (2023). Prospective Life Cycle Assessment of Lithium-Sulfur Batteries for Stationary Energy Storage. ACS Sustainable Chemistry &amp; Engineering. https://doi.org/10.1021/acssuschemeng.3c00141</t>
+        </is>
       </c>
     </row>
     <row r="511" spans="1:11" x14ac:dyDescent="0.2">
@@ -9087,8 +9095,10 @@
         <f>B513</f>
         <v>battery, Li-S</v>
       </c>
-      <c r="H518" t="s">
-        <v>446</v>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>Reference output: 1 kg battery module supplied by this market. The implemented cell reference is 150 Wh/kg cell; at 0.7515918465419887 kg cell/kg module this corresponds to 112.7387769812983 Wh/kg module. The former 321 kg system statement was copied from Li-O2 and is not a Li-S source basis. Quantities and density trajectory unchanged; source-design and equipment-coverage gaps remain unresolved.</t>
+        </is>
       </c>
     </row>
     <row r="519" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>